<commit_message>
Added new RDF data schemes and visual schemes for environment-table09-10, and fixed XLSX spreadsheets for environment-table09-10
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table09.xlsx
+++ b/sources/table_normalization/xlsx/environment-table09.xlsx
@@ -76,9 +76,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
-    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="#,##0.00_ ;\-#,##0.00\ "/>
-    <numFmt numFmtId="169" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00_ ;\-#,##0.00\ "/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -195,10 +195,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -211,10 +211,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -235,7 +235,7 @@
     <xf numFmtId="4" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -251,14 +251,17 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -857,11 +860,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="154509824"/>
-        <c:axId val="147805824"/>
+        <c:axId val="162177024"/>
+        <c:axId val="192484992"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="154509824"/>
+        <c:axId val="162177024"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -899,7 +902,7 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="147805824"/>
+        <c:crossAx val="192484992"/>
         <c:crossesAt val="0"/>
         <c:auto val="0"/>
         <c:lblAlgn val="ctr"/>
@@ -908,7 +911,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="147805824"/>
+        <c:axId val="192484992"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -958,7 +961,7 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="154509824"/>
+        <c:crossAx val="162177024"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1416,11 +1419,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="154510848"/>
-        <c:axId val="147807552"/>
+        <c:axId val="162178048"/>
+        <c:axId val="192486720"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="154510848"/>
+        <c:axId val="162178048"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1458,7 +1461,7 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="147807552"/>
+        <c:crossAx val="192486720"/>
         <c:crossesAt val="0"/>
         <c:auto val="0"/>
         <c:lblAlgn val="ctr"/>
@@ -1467,7 +1470,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="147807552"/>
+        <c:axId val="192486720"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1517,7 +1520,7 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="154510848"/>
+        <c:crossAx val="162178048"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1948,44 +1951,44 @@
       <c r="F3" s="10"/>
     </row>
     <row r="4" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20"/>
-      <c r="B4" s="18" t="s">
+      <c r="A4" s="19"/>
+      <c r="B4" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18" t="s">
+      <c r="C4" s="21"/>
+      <c r="D4" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="18"/>
-      <c r="F4" s="19" t="s">
+      <c r="E4" s="21"/>
+      <c r="F4" s="20" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="20.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
+      <c r="A5" s="19"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
     </row>
     <row r="6" spans="1:6" ht="23.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="20"/>
+      <c r="F6" s="19"/>
     </row>
     <row r="7" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">

</xml_diff>